<commit_message>
Audit Log IP cleaning, DNI for users, and Improved Bulk Upload with progress bar
</commit_message>
<xml_diff>
--- a/front/public/templates/plantilla_carga_masiva.xlsx
+++ b/front/public/templates/plantilla_carga_masiva.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q5"/>
+  <dimension ref="A1:Q6"/>
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -580,52 +580,52 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>P. NACIMIENTO</v>
+        <v>DNI</v>
       </c>
       <c r="B4" s="1" t="str">
-        <v/>
+        <v>30405060</v>
       </c>
       <c r="C4" t="str">
-        <v>BEBE REGISTRADO</v>
+        <v>PEDRO PABLO</v>
       </c>
       <c r="D4" t="str">
-        <v>CUEVA</v>
+        <v>VILLANUEVA</v>
       </c>
       <c r="E4" t="str">
-        <v>SOTO</v>
+        <v>CASTRO</v>
       </c>
       <c r="F4" t="str">
         <v>M</v>
       </c>
       <c r="G4" t="str">
-        <v>2024-02-10</v>
+        <v>1950-01-01</v>
       </c>
       <c r="H4" s="1" t="str">
         <v/>
       </c>
       <c r="I4" t="str">
-        <v>Sin DNI por ser menor</v>
+        <v>Fallecido</v>
       </c>
       <c r="J4" t="str">
-        <v>NACIMIENTO</v>
+        <v>DEFUNCION</v>
       </c>
       <c r="K4" s="1" t="str">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="L4" s="1" t="str">
-        <v>200</v>
+        <v>77</v>
       </c>
       <c r="M4" s="1" t="str">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="N4" t="str">
-        <v>2024-02-28</v>
+        <v>2023-11-20</v>
       </c>
       <c r="O4" t="str">
         <v/>
       </c>
       <c r="P4" t="str">
-        <v>prueba/nacimientos/LIBRO 2</v>
+        <v>prueba/defunciones/LIBRO 1</v>
       </c>
       <c r="Q4" t="str">
         <v>Documento 1.pdf</v>
@@ -633,15 +633,68 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
+        <v>P. NACIMIENTO</v>
+      </c>
+      <c r="B5" s="1" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
+        <v>BEBE REGISTRADO</v>
+      </c>
+      <c r="D5" t="str">
+        <v>CUEVA</v>
+      </c>
+      <c r="E5" t="str">
+        <v>SOTO</v>
+      </c>
+      <c r="F5" t="str">
+        <v>M</v>
+      </c>
+      <c r="G5" t="str">
+        <v>2024-02-10</v>
+      </c>
+      <c r="H5" s="1" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v>Sin DNI por ser menor</v>
+      </c>
+      <c r="J5" t="str">
+        <v>NACIMIENTO</v>
+      </c>
+      <c r="K5" s="1" t="str">
+        <v>5</v>
+      </c>
+      <c r="L5" s="1" t="str">
+        <v>200</v>
+      </c>
+      <c r="M5" s="1" t="str">
+        <v>2024</v>
+      </c>
+      <c r="N5" t="str">
+        <v>2024-02-28</v>
+      </c>
+      <c r="O5" t="str">
+        <v/>
+      </c>
+      <c r="P5" t="str">
+        <v>prueba/nacimientos/LIBRO 2</v>
+      </c>
+      <c r="Q5" t="str">
+        <v>Documento 1.pdf</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
         <v>INSTRUCCIONES: Azul=Ciudadano | Verde=Acta | Amarillo=Archivo PDF (opcional). Fechas en formato AAAA-MM-DD (ej: 1990-05-15). carpeta_ruta = solo la carpeta dentro del ZIP, SIN el nombre del archivo. Ej: prueba/nacimientos/LIBRO 1</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A5:Q5"/>
+    <mergeCell ref="A6:Q6"/>
   </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>